<commit_message>
In the config file for the JV2 script, add the references to the p8 parameters
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\Tutorial6_JV_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3D1D79-C8B2-4DDC-9B73-54A517EAF1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2160762A-0F10-4F1B-91E2-168D758D69E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="148">
   <si>
     <t>Description</t>
   </si>
@@ -466,6 +466,18 @@
   </si>
   <si>
     <t>Share of P5 going to recycling TODO</t>
+  </si>
+  <si>
+    <t>ODYM_T6_P8_BlackmassExport</t>
+  </si>
+  <si>
+    <t>ODYM_T6_P8_RecoveredNotForBattery</t>
+  </si>
+  <si>
+    <t>ODYM_T6_P8_RecycledExport</t>
+  </si>
+  <si>
+    <t>ODYM_T6_P8_RecycledDomesticProduction</t>
   </si>
 </sst>
 </file>
@@ -1211,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J62"/>
+  <dimension ref="B2:J68"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.88671875" customWidth="1"/>
@@ -1960,77 +1972,109 @@
         <v>141</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C49" s="27"/>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B50" s="18" t="s">
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C49" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="I49" s="37"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C50" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="I50" s="37"/>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C51" s="27" t="s">
+        <v>146</v>
+      </c>
+      <c r="I51" s="37"/>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C52" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="I52" s="37"/>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C53" s="27"/>
+      <c r="I53" s="37"/>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C54" s="27"/>
+      <c r="I54" s="37"/>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C55" s="27"/>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B56" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
-      <c r="G50" s="19"/>
-      <c r="H50" s="20"/>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C51" t="s">
+      <c r="C56" s="19"/>
+      <c r="D56" s="19"/>
+      <c r="E56" s="19"/>
+      <c r="F56" s="19"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="20"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C57" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C52" s="27" t="s">
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C58" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="D52" s="33" t="s">
+      <c r="D58" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E58" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D53" s="33"/>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D54" s="33"/>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D55" s="33"/>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D56" s="33"/>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D57" s="33"/>
-    </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B59" s="18" t="s">
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D59" s="33"/>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D60" s="33"/>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D61" s="33"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D62" s="33"/>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D63" s="33"/>
+    </row>
+    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B65" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="20"/>
-    </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C60" t="s">
+      <c r="C65" s="19"/>
+      <c r="D65" s="19"/>
+      <c r="E65" s="19"/>
+      <c r="F65" s="19"/>
+      <c r="G65" s="19"/>
+      <c r="H65" s="20"/>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C66" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B62" s="18" t="s">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B68" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="C62" s="19"/>
-      <c r="D62" s="19"/>
-      <c r="E62" s="19"/>
-      <c r="F62" s="19"/>
-      <c r="G62" s="19"/>
-      <c r="H62" s="20"/>
+      <c r="C68" s="19"/>
+      <c r="D68" s="19"/>
+      <c r="E68" s="19"/>
+      <c r="F68" s="19"/>
+      <c r="G68" s="19"/>
+      <c r="H68" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Changed the process list to have 8 processes to match the flows as described in the flows chunk instead of skipping #1 in the labeling. Also fixed typo in ToLandfillRate file
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\Tutorial6_JV_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2160762A-0F10-4F1B-91E2-168D758D69E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70E67B9-A7B2-4A85-BD4A-9A33E0C0EC4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="156">
   <si>
     <t>Description</t>
   </si>
@@ -408,9 +408,6 @@
     <t>Scenario analysis of dispersion of steel into different applications.</t>
   </si>
   <si>
-    <t>Consider removing if unnecesary for code</t>
-  </si>
-  <si>
     <t>Production</t>
   </si>
   <si>
@@ -420,9 +417,6 @@
     <t>Used battery collection and sorting</t>
   </si>
   <si>
-    <t>Consider reclassifying as Industry</t>
-  </si>
-  <si>
     <t>Landfill</t>
   </si>
   <si>
@@ -432,15 +426,36 @@
     <t>Recycling</t>
   </si>
   <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e6</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e7</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e8</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e9</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c2210</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c2211</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c2212</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c2213</t>
+  </si>
+  <si>
     <t>ODYM_T6_P5_ToLandfillRate</t>
   </si>
   <si>
     <t>Share of P5 going to landfill</t>
   </si>
   <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c22e6</t>
-  </si>
-  <si>
     <t>ODYM_T6_P5_ToUsedExportRate</t>
   </si>
   <si>
@@ -450,41 +465,50 @@
     <t>ODYM_T6_P5_ToRefurbishment</t>
   </si>
   <si>
+    <t>Share of P5 going to refurbishment (currently 0%) TODO</t>
+  </si>
+  <si>
     <t>ODYM_T6_P5_ToRecycling</t>
   </si>
   <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c22e7</t>
-  </si>
-  <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c22e8</t>
-  </si>
-  <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c22e9</t>
-  </si>
-  <si>
-    <t>Share of P5 going to refurbishment (currently 0%) TODO</t>
-  </si>
-  <si>
-    <t>Share of P5 going to recycling TODO</t>
+    <t>Share of P5 going to recycling</t>
   </si>
   <si>
     <t>ODYM_T6_P8_BlackmassExport</t>
   </si>
   <si>
+    <t>Share of P8 going to blackmass export</t>
+  </si>
+  <si>
     <t>ODYM_T6_P8_RecoveredNotForBattery</t>
   </si>
   <si>
+    <t>Share of P8 going to other products</t>
+  </si>
+  <si>
     <t>ODYM_T6_P8_RecycledExport</t>
   </si>
   <si>
+    <t>Share of P8 going to recycled battery material for export</t>
+  </si>
+  <si>
     <t>ODYM_T6_P8_RecycledDomesticProduction</t>
+  </si>
+  <si>
+    <t>Share of P8 going to recycled battery material for domestic production</t>
+  </si>
+  <si>
+    <t>Extraction</t>
+  </si>
+  <si>
+    <t>Unused in this example</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -552,6 +576,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -1223,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J68"/>
+  <dimension ref="B2:J69"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.88671875" customWidth="1"/>
@@ -1627,74 +1657,71 @@
       <c r="E28" t="s">
         <v>85</v>
       </c>
-      <c r="F28" t="s">
-        <v>124</v>
-      </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C29" s="31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>125</v>
+        <v>154</v>
       </c>
       <c r="E29" t="s">
         <v>54</v>
       </c>
+      <c r="F29" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C30" s="27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C31" s="27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="E31" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C32" s="31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>127</v>
+        <v>34</v>
       </c>
       <c r="E32" t="s">
-        <v>55</v>
-      </c>
-      <c r="F32" t="s">
-        <v>128</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C33" s="27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E33" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C34" s="31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E34" t="s">
         <v>54</v>
@@ -1702,107 +1729,95 @@
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C35" s="27">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E35" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B37" s="18" t="s">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C36" s="27">
+        <v>8</v>
+      </c>
+      <c r="D36" t="s">
+        <v>129</v>
+      </c>
+      <c r="E36" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B38" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="20"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C38" s="26" t="s">
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="20"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C39" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="23" t="s">
+      <c r="D39" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="E39" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="F38" s="23" t="s">
+      <c r="F39" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="G38" s="23" t="s">
+      <c r="G39" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H38" s="23" t="s">
+      <c r="H39" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="I38" s="36" t="s">
+      <c r="I39" s="36" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C39" t="s">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C40" t="s">
         <v>98</v>
       </c>
-      <c r="D39" s="38" t="s">
+      <c r="D40" s="38" t="s">
         <v>83</v>
-      </c>
-      <c r="E39" t="s">
-        <v>97</v>
-      </c>
-      <c r="F39" t="s">
-        <v>61</v>
-      </c>
-      <c r="G39" t="s">
-        <v>31</v>
-      </c>
-      <c r="H39" t="s">
-        <v>31</v>
-      </c>
-      <c r="I39" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C40" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="D40" t="s">
-        <v>104</v>
       </c>
       <c r="E40" t="s">
         <v>97</v>
       </c>
       <c r="F40" t="s">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="G40" t="s">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="H40" t="s">
         <v>31</v>
       </c>
       <c r="I40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C41" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D41" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E41" t="s">
         <v>97</v>
       </c>
       <c r="F41" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G41" t="s">
         <v>78</v>
@@ -1810,16 +1825,16 @@
       <c r="H41" t="s">
         <v>31</v>
       </c>
-      <c r="I41" s="37" t="s">
-        <v>103</v>
+      <c r="I41" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C42" s="27" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D42" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E42" t="s">
         <v>97</v>
@@ -1834,41 +1849,44 @@
         <v>31</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C43" s="27" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D43" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E43" t="s">
         <v>97</v>
       </c>
       <c r="F43" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="G43" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H43" t="s">
         <v>31</v>
       </c>
       <c r="I43" s="37" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C44" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
+      </c>
+      <c r="D44" t="s">
+        <v>116</v>
       </c>
       <c r="E44" t="s">
         <v>97</v>
       </c>
       <c r="F44" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G44" t="s">
         <v>84</v>
@@ -1877,38 +1895,35 @@
         <v>31</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="D45" t="s">
-        <v>133</v>
+        <v>112</v>
       </c>
       <c r="E45" t="s">
         <v>97</v>
       </c>
       <c r="F45" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="G45" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="H45" t="s">
         <v>31</v>
       </c>
       <c r="I45" s="37" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C46" s="27" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D46" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E46" t="s">
         <v>97</v>
@@ -1923,15 +1938,15 @@
         <v>31</v>
       </c>
       <c r="I46" s="37" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C47" s="27" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D47" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E47" t="s">
         <v>97</v>
@@ -1946,12 +1961,12 @@
         <v>31</v>
       </c>
       <c r="I47" s="37" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C48" s="27" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
         <v>143</v>
@@ -1969,36 +1984,123 @@
         <v>31</v>
       </c>
       <c r="I48" s="37" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C49" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="I49" s="37"/>
+      <c r="D49" t="s">
+        <v>145</v>
+      </c>
+      <c r="E49" t="s">
+        <v>97</v>
+      </c>
+      <c r="F49" t="s">
+        <v>106</v>
+      </c>
+      <c r="G49" t="s">
+        <v>78</v>
+      </c>
+      <c r="H49" t="s">
+        <v>31</v>
+      </c>
+      <c r="I49" s="37" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C50" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="I50" s="37"/>
+        <v>146</v>
+      </c>
+      <c r="D50" t="s">
+        <v>147</v>
+      </c>
+      <c r="E50" t="s">
+        <v>97</v>
+      </c>
+      <c r="F50" t="s">
+        <v>106</v>
+      </c>
+      <c r="G50" t="s">
+        <v>78</v>
+      </c>
+      <c r="H50" t="s">
+        <v>31</v>
+      </c>
+      <c r="I50" s="37" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C51" s="27" t="s">
-        <v>146</v>
-      </c>
-      <c r="I51" s="37"/>
+        <v>148</v>
+      </c>
+      <c r="D51" t="s">
+        <v>149</v>
+      </c>
+      <c r="E51" t="s">
+        <v>97</v>
+      </c>
+      <c r="F51" t="s">
+        <v>106</v>
+      </c>
+      <c r="G51" t="s">
+        <v>78</v>
+      </c>
+      <c r="H51" t="s">
+        <v>31</v>
+      </c>
+      <c r="I51" s="37" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C52" s="27" t="s">
-        <v>147</v>
-      </c>
-      <c r="I52" s="37"/>
+        <v>150</v>
+      </c>
+      <c r="D52" t="s">
+        <v>151</v>
+      </c>
+      <c r="E52" t="s">
+        <v>97</v>
+      </c>
+      <c r="F52" t="s">
+        <v>106</v>
+      </c>
+      <c r="G52" t="s">
+        <v>78</v>
+      </c>
+      <c r="H52" t="s">
+        <v>31</v>
+      </c>
+      <c r="I52" s="37" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C53" s="27"/>
-      <c r="I53" s="37"/>
+      <c r="C53" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="D53" t="s">
+        <v>153</v>
+      </c>
+      <c r="E53" t="s">
+        <v>97</v>
+      </c>
+      <c r="F53" t="s">
+        <v>106</v>
+      </c>
+      <c r="G53" t="s">
+        <v>78</v>
+      </c>
+      <c r="H53" t="s">
+        <v>31</v>
+      </c>
+      <c r="I53" s="37" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C54" s="27"/>
@@ -2006,36 +2108,37 @@
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C55" s="27"/>
+      <c r="I55" s="37"/>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B56" s="18" t="s">
+      <c r="C56" s="27"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B57" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C56" s="19"/>
-      <c r="D56" s="19"/>
-      <c r="E56" s="19"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="20"/>
-    </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C57" t="s">
+      <c r="C57" s="19"/>
+      <c r="D57" s="19"/>
+      <c r="E57" s="19"/>
+      <c r="F57" s="19"/>
+      <c r="G57" s="19"/>
+      <c r="H57" s="20"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C58" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C58" s="27" t="s">
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C59" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="D58" s="33" t="s">
+      <c r="D59" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E59" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D59" s="33"/>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D60" s="33"/>
@@ -2049,34 +2152,38 @@
     <row r="63" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D63" s="33"/>
     </row>
-    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B65" s="18" t="s">
+    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D64" s="33"/>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B66" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C65" s="19"/>
-      <c r="D65" s="19"/>
-      <c r="E65" s="19"/>
-      <c r="F65" s="19"/>
-      <c r="G65" s="19"/>
-      <c r="H65" s="20"/>
-    </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C66" t="s">
+      <c r="C66" s="19"/>
+      <c r="D66" s="19"/>
+      <c r="E66" s="19"/>
+      <c r="F66" s="19"/>
+      <c r="G66" s="19"/>
+      <c r="H66" s="20"/>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C67" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B68" s="18" t="s">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B69" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="C68" s="19"/>
-      <c r="D68" s="19"/>
-      <c r="E68" s="19"/>
-      <c r="F68" s="19"/>
-      <c r="G68" s="19"/>
-      <c r="H68" s="20"/>
+      <c r="C69" s="19"/>
+      <c r="D69" s="19"/>
+      <c r="E69" s="19"/>
+      <c r="F69" s="19"/>
+      <c r="G69" s="19"/>
+      <c r="H69" s="20"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
in add refernces to parameter files in ODYM_Config_Tutorial6.xlsx
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\Tutorial6_JV_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70E67B9-A7B2-4A85-BD4A-9A33E0C0EC4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706C029A-C01D-4DD9-A2A7-BD086DF26F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="162">
   <si>
     <t>Description</t>
   </si>
@@ -502,6 +502,24 @@
   </si>
   <si>
     <t>Unused in this example</t>
+  </si>
+  <si>
+    <t>ODYM_T7_P3_RefurbishedRate</t>
+  </si>
+  <si>
+    <t>Share of P7 going to re-sale</t>
+  </si>
+  <si>
+    <t>ODYM_T7_P3_RefurbishedLoss</t>
+  </si>
+  <si>
+    <t>Share of P7 material loss</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c2214</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c2215</t>
   </si>
 </sst>
 </file>
@@ -1253,7 +1271,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J69"/>
+  <dimension ref="B2:J70"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.88671875" customWidth="1"/>
@@ -2103,45 +2121,84 @@
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C54" s="27"/>
-      <c r="I54" s="37"/>
+      <c r="C54" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="D54" t="s">
+        <v>157</v>
+      </c>
+      <c r="E54" t="s">
+        <v>97</v>
+      </c>
+      <c r="F54" t="s">
+        <v>106</v>
+      </c>
+      <c r="G54" t="s">
+        <v>78</v>
+      </c>
+      <c r="H54" t="s">
+        <v>31</v>
+      </c>
+      <c r="I54" s="37" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C55" s="27"/>
-      <c r="I55" s="37"/>
+      <c r="C55" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="D55" t="s">
+        <v>159</v>
+      </c>
+      <c r="E55" t="s">
+        <v>97</v>
+      </c>
+      <c r="F55" t="s">
+        <v>106</v>
+      </c>
+      <c r="G55" t="s">
+        <v>78</v>
+      </c>
+      <c r="H55" t="s">
+        <v>31</v>
+      </c>
+      <c r="I55" s="37" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C56" s="27"/>
+      <c r="I56" s="37"/>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B57" s="18" t="s">
+      <c r="C57" s="27"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B58" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="19"/>
-      <c r="H57" s="20"/>
-    </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C58" t="s">
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="20"/>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C59" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C59" s="27" t="s">
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C60" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="D59" s="33" t="s">
+      <c r="D60" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E60" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D60" s="33"/>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D61" s="33"/>
@@ -2155,32 +2212,35 @@
     <row r="64" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D64" s="33"/>
     </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B66" s="18" t="s">
+    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D65" s="33"/>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B67" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C66" s="19"/>
-      <c r="D66" s="19"/>
-      <c r="E66" s="19"/>
-      <c r="F66" s="19"/>
-      <c r="G66" s="19"/>
-      <c r="H66" s="20"/>
-    </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C67" t="s">
+      <c r="C67" s="19"/>
+      <c r="D67" s="19"/>
+      <c r="E67" s="19"/>
+      <c r="F67" s="19"/>
+      <c r="G67" s="19"/>
+      <c r="H67" s="20"/>
+    </row>
+    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C68" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B69" s="18" t="s">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B70" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="C69" s="19"/>
-      <c r="D69" s="19"/>
-      <c r="E69" s="19"/>
-      <c r="F69" s="19"/>
-      <c r="G69" s="19"/>
-      <c r="H69" s="20"/>
+      <c r="C70" s="19"/>
+      <c r="D70" s="19"/>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="20"/>
     </row>
   </sheetData>
   <phoneticPr fontId="11" type="noConversion"/>

</xml_diff>

<commit_message>
Restore the ODYM_Config_Tutorial6 file to before adding the references to P7 parameter files to align with last tested state of the script up to Step 3. Changes will be kept in JV_branch
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\Tutorial6_JV_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706C029A-C01D-4DD9-A2A7-BD086DF26F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A5C950F-10F0-4D21-8522-0BD276C26C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="156">
   <si>
     <t>Description</t>
   </si>
@@ -502,24 +502,6 @@
   </si>
   <si>
     <t>Unused in this example</t>
-  </si>
-  <si>
-    <t>ODYM_T7_P3_RefurbishedRate</t>
-  </si>
-  <si>
-    <t>Share of P7 going to re-sale</t>
-  </si>
-  <si>
-    <t>ODYM_T7_P3_RefurbishedLoss</t>
-  </si>
-  <si>
-    <t>Share of P7 material loss</t>
-  </si>
-  <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c2214</t>
-  </si>
-  <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c2215</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J70"/>
+  <dimension ref="B2:J68"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.88671875" customWidth="1"/>
@@ -2121,84 +2103,44 @@
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C54" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="D54" t="s">
-        <v>157</v>
-      </c>
-      <c r="E54" t="s">
-        <v>97</v>
-      </c>
-      <c r="F54" t="s">
-        <v>106</v>
-      </c>
-      <c r="G54" t="s">
-        <v>78</v>
-      </c>
-      <c r="H54" t="s">
-        <v>31</v>
-      </c>
-      <c r="I54" s="37" t="s">
-        <v>160</v>
-      </c>
+      <c r="C54" s="27"/>
+      <c r="I54" s="37"/>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C55" s="27" t="s">
-        <v>158</v>
-      </c>
-      <c r="D55" t="s">
-        <v>159</v>
-      </c>
-      <c r="E55" t="s">
-        <v>97</v>
-      </c>
-      <c r="F55" t="s">
-        <v>106</v>
-      </c>
-      <c r="G55" t="s">
-        <v>78</v>
-      </c>
-      <c r="H55" t="s">
-        <v>31</v>
-      </c>
-      <c r="I55" s="37" t="s">
-        <v>161</v>
-      </c>
+      <c r="C55" s="27"/>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C56" s="27"/>
-      <c r="I56" s="37"/>
+      <c r="B56" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C56" s="19"/>
+      <c r="D56" s="19"/>
+      <c r="E56" s="19"/>
+      <c r="F56" s="19"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="20"/>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C57" s="27"/>
+      <c r="C57" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B58" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="20"/>
+      <c r="C58" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="D58" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="E58" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C59" t="s">
-        <v>42</v>
-      </c>
+      <c r="D59" s="33"/>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C60" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="D60" s="33" t="s">
-        <v>44</v>
-      </c>
-      <c r="E60" t="s">
-        <v>45</v>
-      </c>
+      <c r="D60" s="33"/>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D61" s="33"/>
@@ -2209,38 +2151,32 @@
     <row r="63" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D63" s="33"/>
     </row>
-    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="D64" s="33"/>
-    </row>
     <row r="65" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D65" s="33"/>
-    </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B67" s="18" t="s">
+      <c r="B65" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C67" s="19"/>
-      <c r="D67" s="19"/>
-      <c r="E67" s="19"/>
-      <c r="F67" s="19"/>
-      <c r="G67" s="19"/>
-      <c r="H67" s="20"/>
+      <c r="C65" s="19"/>
+      <c r="D65" s="19"/>
+      <c r="E65" s="19"/>
+      <c r="F65" s="19"/>
+      <c r="G65" s="19"/>
+      <c r="H65" s="20"/>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C66" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="68" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C68" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B70" s="18" t="s">
+      <c r="B68" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="C70" s="19"/>
-      <c r="D70" s="19"/>
-      <c r="E70" s="19"/>
-      <c r="F70" s="19"/>
-      <c r="G70" s="19"/>
-      <c r="H70" s="20"/>
+      <c r="C68" s="19"/>
+      <c r="D68" s="19"/>
+      <c r="E68" s="19"/>
+      <c r="F68" s="19"/>
+      <c r="G68" s="19"/>
+      <c r="H68" s="20"/>
     </row>
   </sheetData>
   <phoneticPr fontId="11" type="noConversion"/>

</xml_diff>

<commit_message>
Add rates for refurbishment and refurbishment material losss, both should sum to 1
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\Tutorial6_JV_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706C029A-C01D-4DD9-A2A7-BD086DF26F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F333D15B-CE88-4738-A44E-E71B4DA0946D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -504,15 +504,9 @@
     <t>Unused in this example</t>
   </si>
   <si>
-    <t>ODYM_T7_P3_RefurbishedRate</t>
-  </si>
-  <si>
     <t>Share of P7 going to re-sale</t>
   </si>
   <si>
-    <t>ODYM_T7_P3_RefurbishedLoss</t>
-  </si>
-  <si>
     <t>Share of P7 material loss</t>
   </si>
   <si>
@@ -520,6 +514,12 @@
   </si>
   <si>
     <t>6213e899-8367-483a-8d09-a0c0831c2215</t>
+  </si>
+  <si>
+    <t>ODYM_T6_P7_RefurbishedRate</t>
+  </si>
+  <si>
+    <t>ODYM_T6_P7_RefurbishedLossRate</t>
   </si>
 </sst>
 </file>
@@ -2122,10 +2122,10 @@
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C54" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="D54" t="s">
         <v>156</v>
-      </c>
-      <c r="D54" t="s">
-        <v>157</v>
       </c>
       <c r="E54" t="s">
         <v>97</v>
@@ -2140,15 +2140,15 @@
         <v>31</v>
       </c>
       <c r="I54" s="37" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C55" s="27" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D55" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E55" t="s">
         <v>97</v>
@@ -2163,7 +2163,7 @@
         <v>31</v>
       </c>
       <c r="I55" s="37" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updates, reverting to version before changes made
</commit_message>
<xml_diff>
--- a/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
+++ b/docs/Files/Tutorial6_JV_2/ODYM_Config_Tutorial6.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\Tutorial6_JV_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elanphear\Code\ODYM\docs\Files\Tutorial6_JV_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70E67B9-A7B2-4A85-BD4A-9A33E0C0EC4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC597341-3B61-4B78-A48F-BD4E1D45E2AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="5" r:id="rId1"/>
@@ -1070,14 +1070,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5546875" customWidth="1"/>
+    <col min="4" max="4" width="26.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B1" s="29" t="s">
         <v>37</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="6"/>
       <c r="B2" s="8" t="s">
         <v>39</v>
@@ -1095,12 +1095,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="6"/>
       <c r="B3" s="8"/>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="6"/>
       <c r="B4" s="9" t="s">
         <v>2</v>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="G4" s="35"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="6"/>
       <c r="B5" s="9" t="s">
         <v>52</v>
@@ -1125,122 +1125,122 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="6"/>
       <c r="B6" s="9"/>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="6"/>
       <c r="B7" s="9"/>
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="6"/>
       <c r="B8" s="9"/>
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="6"/>
       <c r="B9" s="11"/>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="10"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="10"/>
       <c r="B11" s="12"/>
       <c r="C11" s="14"/>
       <c r="D11" s="12"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="10"/>
       <c r="B12" s="12"/>
       <c r="C12" s="15"/>
       <c r="D12" s="12"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="10"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="10"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="10"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="10"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="10"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="10"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="10"/>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="10"/>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="10"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="10"/>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="10"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="6"/>
       <c r="B25" s="1"/>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="1"/>
       <c r="C26" s="2"/>
@@ -1254,19 +1254,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:J69"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="4.88671875" customWidth="1"/>
+    <col min="2" max="2" width="4.90625" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="44.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.6640625" customWidth="1"/>
-    <col min="6" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6328125" customWidth="1"/>
+    <col min="6" max="6" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.36328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B2" s="18" t="s">
         <v>3</v>
       </c>
@@ -1277,7 +1277,7 @@
       <c r="G2" s="19"/>
       <c r="H2" s="20"/>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C3" s="23" t="s">
         <v>27</v>
       </c>
@@ -1289,7 +1289,7 @@
       <c r="G3" s="30"/>
       <c r="H3" s="30"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>4</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>0</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>5</v>
       </c>
@@ -1313,11 +1313,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D7" s="7"/>
       <c r="J7" s="13"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8" s="18" t="s">
         <v>40</v>
       </c>
@@ -1329,7 +1329,7 @@
       <c r="H8" s="20"/>
       <c r="J8" s="13"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C9" s="23" t="s">
         <v>27</v>
       </c>
@@ -1344,7 +1344,7 @@
       <c r="H9" s="30"/>
       <c r="J9" s="13"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>6</v>
       </c>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="J10" s="13"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>57</v>
       </c>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="J11" s="13"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>58</v>
       </c>
@@ -1371,10 +1371,10 @@
       </c>
       <c r="J12" s="13"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
       <c r="J13" s="17"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
         <v>50</v>
       </c>
@@ -1387,7 +1387,7 @@
       <c r="G14" s="19"/>
       <c r="H14" s="20"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C15" s="24" t="s">
         <v>7</v>
       </c>
@@ -1413,7 +1413,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C16" s="25" t="s">
         <v>11</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C17" s="25" t="s">
         <v>73</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C18" s="25" t="s">
         <v>15</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C19" s="25" t="s">
         <v>16</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C20" s="25" t="s">
         <v>79</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C21" s="25" t="s">
         <v>60</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C22" s="25" t="s">
         <v>12</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C23" s="25" t="s">
         <v>14</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C24" s="21" t="s">
         <v>91</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>46</v>
       </c>
@@ -1631,7 +1631,7 @@
       <c r="G26" s="19"/>
       <c r="H26" s="20"/>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C27" s="26" t="s">
         <v>47</v>
       </c>
@@ -1647,7 +1647,7 @@
       <c r="G27" s="30"/>
       <c r="H27" s="30"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C28" s="31">
         <v>0</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C29" s="31">
         <v>1</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C30" s="27">
         <v>2</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C31" s="27">
         <v>3</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C32" s="31">
         <v>4</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C33" s="27">
         <v>5</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C34" s="31">
         <v>6</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C35" s="27">
         <v>7</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C36" s="27">
         <v>8</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B38" s="18" t="s">
         <v>25</v>
       </c>
@@ -1760,7 +1760,7 @@
       <c r="G38" s="19"/>
       <c r="H38" s="20"/>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C39" s="26" t="s">
         <v>28</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C40" t="s">
         <v>98</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C41" s="27" t="s">
         <v>101</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C42" s="27" t="s">
         <v>102</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C43" s="27" t="s">
         <v>110</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C44" s="27" t="s">
         <v>113</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C45" s="27" t="s">
         <v>112</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C46" s="27" t="s">
         <v>138</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C47" s="27" t="s">
         <v>140</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C48" s="27" t="s">
         <v>142</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C49" s="27" t="s">
         <v>144</v>
       </c>
@@ -2010,7 +2010,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C50" s="27" t="s">
         <v>146</v>
       </c>
@@ -2033,7 +2033,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C51" s="27" t="s">
         <v>148</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C52" s="27" t="s">
         <v>150</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C53" s="27" t="s">
         <v>152</v>
       </c>
@@ -2102,18 +2102,18 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C54" s="27"/>
       <c r="I54" s="37"/>
     </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C55" s="27"/>
       <c r="I55" s="37"/>
     </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C56" s="27"/>
     </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B57" s="18" t="s">
         <v>41</v>
       </c>
@@ -2124,12 +2124,12 @@
       <c r="G57" s="19"/>
       <c r="H57" s="20"/>
     </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C58" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C59" s="27" t="s">
         <v>43</v>
       </c>
@@ -2140,22 +2140,22 @@
         <v>45</v>
       </c>
     </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:9" x14ac:dyDescent="0.35">
       <c r="D60" s="33"/>
     </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:9" x14ac:dyDescent="0.35">
       <c r="D61" s="33"/>
     </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:9" x14ac:dyDescent="0.35">
       <c r="D62" s="33"/>
     </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:9" x14ac:dyDescent="0.35">
       <c r="D63" s="33"/>
     </row>
-    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:9" x14ac:dyDescent="0.35">
       <c r="D64" s="33"/>
     </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B66" s="18" t="s">
         <v>49</v>
       </c>
@@ -2166,12 +2166,12 @@
       <c r="G66" s="19"/>
       <c r="H66" s="20"/>
     </row>
-    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C67" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B69" s="18" t="s">
         <v>119</v>
       </c>

</xml_diff>